<commit_message>
docs: seal verified Windows build, CI results and test access delivery
</commit_message>
<xml_diff>
--- a/outputs/01a15734-c809-7ff2-8313-f617805a4441/部署手册及打包清单.xlsx
+++ b/outputs/01a15734-c809-7ff2-8313-f617805a4441/部署手册及打包清单.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="部署总览" sheetId="1" r:id="Rdcea5865463c443f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境配置" sheetId="2" r:id="R0b6ab53de96a4f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布与回退步骤" sheetId="3" r:id="R8232cbbc65994dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="打包文件清单" sheetId="4" r:id="R4d2264fd7a054ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实际归档文件" sheetId="5" r:id="R557a3565f3f24a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控与运维" sheetId="6" r:id="Rfd08d2d1e4894156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付与阻塞" sheetId="7" r:id="Rffc80fdcbff047b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="部署总览" sheetId="1" r:id="Rbae20a8d3f4f49f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="环境配置" sheetId="2" r:id="R4d9f2bcf9ebb43e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布与回退步骤" sheetId="3" r:id="Ra4b943b81f044141"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="打包文件清单" sheetId="4" r:id="R0e4cd4c857774c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实际归档文件" sheetId="5" r:id="Rf9426332fd894e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="监控与运维" sheetId="6" r:id="Rea10df98c5b64a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付与阻塞" sheetId="7" r:id="R33a127d9aebe4ee3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,8 +154,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DesignTable24" displayName="DesignTable24" ref="A5:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DesignTable24" displayName="DesignTable24" ref="A5:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F25"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="包类型"/>
     <x:tableColumn id="2" name="路径或文件"/>
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DesignTable27" displayName="DesignTable27" ref="A5:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DesignTable27" displayName="DesignTable27" ref="A5:E16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E16"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="事项"/>
     <x:tableColumn id="2" name="当前结果"/>
@@ -495,7 +495,7 @@
         <x:v>pyproject.toml:1</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="27" customHeight="1">
+    <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>Launcher</x:v>
       </x:c>
@@ -503,7 +503,7 @@
         <x:v>保留React+Tauri，新增自包含开发包脚本</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Mac未生成Windows归档；正式安装未验收</x:v>
+        <x:v>37b7598 Windows开发包已构建，冻结bootstrap/close烟测通过；实际API/干净安装/实玩未验收</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
         <x:v>玩家包用HTTPS网关或已存在的本机隧道，不附私人SSH配置</x:v>
@@ -585,22 +585,22 @@
         <x:v>远端与CI</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>Git远端未更新；WindowsCI未执行</x:v>
+        <x:v>已推送 origin/fix/launcher-portal-admin</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>推送被自动审批拒绝，待明确目的地授权</x:v>
+        <x:v>Windows工具/前端及MySQL综合检查成功；Launcher构建与冻结烟测成功</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>当前未进行远端Web或Windows部署，不在本任务重试推送</x:v>
+        <x:v>当前未进行远端Web或Windows部署；CI构建不等于安装或游戏验收</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
-        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md:1</x:v>
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R246219e8a4a14c8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ab8916c926847e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -855,7 +855,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c12c4188054450d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10ba389c7ec4111"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1131,7 +1131,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R224b1cd3af2445c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfae2e8bbe574495d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1424,7 +1424,7 @@
         <x:v>tools/monitor_agent.py:1</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="27" customHeight="1">
+    <x:row r="17" ht="36" customHeight="1">
       <x:c r="A17" s="10" t="str">
         <x:v>Launcher开发包</x:v>
       </x:c>
@@ -1435,10 +1435,10 @@
         <x:v>Tauri窗口与公开API设置</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>Windows实际构建后生成</x:v>
+        <x:v>Windows CI已产包；754个payload和manifest独立核验通过</x:v>
       </x:c>
       <x:c r="E17" s="10" t="str">
-        <x:v>未生成Windows zip；配置不允许包含私人SSH/数据库秘密</x:v>
+        <x:v>配置不允许包含私人SSH/数据库秘密；实际CI产物状态见交付与阻塞页</x:v>
       </x:c>
       <x:c r="F17" s="10" t="str">
         <x:v>tools/package_launcher.py:1</x:v>
@@ -1464,7 +1464,7 @@
         <x:v>tools/package_launcher.py:1</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="27" customHeight="1">
+    <x:row r="19" ht="36" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>Launcher开发包</x:v>
       </x:c>
@@ -1475,7 +1475,7 @@
         <x:v>文件字节/摘要、依赖许可、使用边界</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
-        <x:v>Windows实际构建后生成</x:v>
+        <x:v>Windows CI已产包；754个payload和manifest独立核验通过</x:v>
       </x:c>
       <x:c r="E19" s="10" t="str">
         <x:v>manifest内native_start_available=false，PACKAGE_NATIVE_CLIENT_UNAVAILABLE</x:v>
@@ -1484,90 +1484,130 @@
         <x:v>tools/package_launcher.py:1</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="27" customHeight="1">
+    <x:row r="20" ht="36" customHeight="1">
       <x:c r="A20" s="10" t="str">
-        <x:v>原生研究工作区</x:v>
+        <x:v>Launcher实际归档</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>launcher/bin/components/d3d9-frame-copy.dll</x:v>
+        <x:v>NZLauncher-DEV.zip</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
-        <x:v>已有本机原生研究路径的固定摘要x86显示桥</x:v>
+        <x:v>25974212 bytes；SHA256 139c84de2b034d33be4f5079be6821d582112c02d4552b375733f02494102993</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>非本次自包含门户包必要组件</x:v>
+        <x:v>CI产物已独立核验</x:v>
       </x:c>
       <x:c r="E20" s="10" t="str">
-        <x:v>自包含包未带原生客户端，不能声明可以完整游戏启动</x:v>
+        <x:v>754个payload另加manifest；逐文件SHA、路径、排除私密及外置manifest一致性独立核验通过</x:v>
       </x:c>
       <x:c r="F20" s="10" t="str">
-        <x:v>tools/native_frame_bridge.py:1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="27" customHeight="1">
+        <x:v>evidence/2026-10-19-windows-package-verification.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
       <x:c r="A21" s="10" t="str">
-        <x:v>Launcher构建入口</x:v>
+        <x:v>GitHub下载包装层</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>python -m tools.package_launcher --api-base-url https://公开API</x:v>
+        <x:v>https://github.com/016-ops/NZ/actions/runs/39375681700/artifacts/12243650799</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
-        <x:v>生成NZLauncher-DEV目录及同级zip</x:v>
+        <x:v>25777855 bytes；SHA256 d92596490ed233ea21c7102c221449430f2a787d70ee9bf464623e7b71bb25c4</x:v>
       </x:c>
       <x:c r="D21" s="10" t="str">
-        <x:v>Windows执行；--plan可静态审查</x:v>
+        <x:v>artifact wrapper单独摘要</x:v>
       </x:c>
       <x:c r="E21" s="10" t="str">
-        <x:v>已存在输出拒绝覆盖；归档SHA只在实际生成后报告</x:v>
+        <x:v>此摘要属于下载包装层，不能代替NZLauncher-DEV.zip内部发行归档摘要</x:v>
       </x:c>
       <x:c r="F21" s="10" t="str">
-        <x:v>tools/package_launcher.py:1</x:v>
+        <x:v>evidence/2026-10-19-windows-package-verification.json</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
       <x:c r="A22" s="10" t="str">
-        <x:v>排除</x:v>
+        <x:v>原生研究工作区</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>runtime/、evidence/private/、.env*、*.pem、*.key</x:v>
+        <x:v>launcher/bin/components/d3d9-frame-copy.dll</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
-        <x:v>凭据、缓存及私人证据</x:v>
+        <x:v>已有本机原生研究路径的固定摘要x86显示桥</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>必须排除</x:v>
+        <x:v>非本次自包含门户包必要组件</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
-        <x:v>不把排除目录作为游戏安装包依赖分发</x:v>
+        <x:v>自包含包未带原生客户端，不能声明可以完整游戏启动</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
-        <x:v>.gitignore:1</x:v>
+        <x:v>tools/native_frame_bridge.py:1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="27" customHeight="1">
       <x:c r="A23" s="10" t="str">
+        <x:v>Launcher构建入口</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>python -m tools.package_launcher --api-base-url https://公开API</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>生成NZLauncher-DEV目录及同级zip</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>Windows执行；--plan可静态审查</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>已存在输出拒绝覆盖；归档SHA只在实际生成后报告</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="str">
+        <x:v>tools/package_launcher.py:1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="27" customHeight="1">
+      <x:c r="A24" s="10" t="str">
         <x:v>排除</x:v>
       </x:c>
-      <x:c r="B23" s="10" t="str">
+      <x:c r="B24" s="10" t="str">
+        <x:v>runtime/、evidence/private/、.env*、*.pem、*.key</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>凭据、缓存及私人证据</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>必须排除</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>不把排除目录作为游戏安装包依赖分发</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>.gitignore:1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="A25" s="10" t="str">
+        <x:v>排除</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="str">
         <x:v>原始游戏客户端、数据库、node_modules、.git</x:v>
       </x:c>
-      <x:c r="C23" s="10" t="str">
+      <x:c r="C25" s="10" t="str">
         <x:v>第三方大体积数据与源码管理内部信息</x:v>
       </x:c>
-      <x:c r="D23" s="10" t="str">
+      <x:c r="D25" s="10" t="str">
         <x:v>必须排除</x:v>
       </x:c>
-      <x:c r="E23" s="10" t="str">
+      <x:c r="E25" s="10" t="str">
         <x:v>游戏内容分发与授权单独安排</x:v>
       </x:c>
-      <x:c r="F23" s="10" t="str">
+      <x:c r="F25" s="10" t="str">
         <x:v>.gitignore:1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ccf29e5891d4e34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae2e3630ef4b474d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4440,7 +4480,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R636c9d1b152c4660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bea6261f7624164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4678,7 +4718,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbc3e5f4a389400a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c75188f0ca64563"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4760,18 +4800,18 @@
         <x:v>docs/WEB_DEPLOYMENT.md:1</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="27" customHeight="1">
+    <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>Windows开发包</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>继续现有Tauri构建，不部署远端Windows</x:v>
+        <x:v>37b7598 Windows开发包已构建，冻结bootstrap/close烟测通过；实际API/干净安装/实玩未验收</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>正式签名、干净安装和受限玩家网关另验</x:v>
+        <x:v>默认回环18765占位需改正式网关；API登录、正式签名、干净Windows安装及实玩另验</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>安装/卸载/升级/退出恢复及无秘密分发</x:v>
+        <x:v>安装/卸载/升级/退出恢复及无秘密分发；CI不代替实际安装验收</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
         <x:v>docs/native-launcher.md:1</x:v>
@@ -4850,39 +4890,90 @@
         <x:v>Git提交与推送</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>实现已本地提交；远端未更新</x:v>
+        <x:v>已推送 origin/fix/launcher-portal-admin</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>自动审批拒绝外部GitHub推送，目的地待用户明确授权</x:v>
+        <x:v>用户已明确授权并完成GitHub认证；推送成功，ls-remote与本地推送提交一致</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>不得把本地提交说成远端已更新；不重试未获授权推送</x:v>
+        <x:v>6f12054997e32258e807980265dad04a4afe914e</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
-        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md:1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="27" customHeight="1">
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="50" customHeight="1">
       <x:c r="A13" s="10" t="str">
-        <x:v>WindowsCI</x:v>
+        <x:v>Launcher构建CI</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>未执行</x:v>
+        <x:v>success：构建与冻结bootstrap/close烟测通过</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>本机Mac仅验证脚本/界面与Linux兼容工具</x:v>
+        <x:v>37b7598；artifact12243650799已上传，innerZip的754个payload及manifest路径/摘要/排除私密/外置清单一致性已独立核验。未连接实际API、未干净Windows安装、未实玩；默认回环18765仍为占位网关</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>实际Windows产包、签名、安装/升级与干净机器验收另记</x:v>
+        <x:v>https://github.com/016-ops/NZ/actions/runs/39375681700</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
-        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md:1</x:v>
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="36" customHeight="1">
+      <x:c r="A14" s="10" t="str">
+        <x:v>Windows工具/前端CI</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>工具/前端job成功</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>6f12054：246项、245通过、0失败/错误、2.748秒；1项测试内skip及6个缺原件suite skip另列，不混进实际通过数；前端成功</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>https://github.com/016-ops/NZ/actions/runs/39375957208/job/118474030815</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="10" t="str">
+        <x:v>综合CI</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>success：MySQL及Windows两个job成功</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>6f12054，MySQL8.4.11：579项、565通过、0失败/错误、582.514秒；14项测试内Skip及6个缺原件suite Skip单列，不计为通过；未据此声称Windows-only场景全部已验证</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>https://github.com/016-ops/NZ/actions/runs/39375957208</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="27" customHeight="1">
+      <x:c r="A16" s="10" t="str">
+        <x:v>本机演示账号</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>test-player@example.invalid / nz-test-admin</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Owner使用正常MFA；凭据仅存本机runtime私密文件，未写入Excel或发布包</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>http://127.0.0.1:8875/player / http://127.0.0.1:8875/admin；隔离演示账号已创建，仅供本机验证</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>docs/delivery/2026-10-19-launcher-portal-admin.md:125</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R422f4b12bac44239"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31948a9df909409e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>